<commit_message>
added more robust easing function for calculating penalty for the previous winners
</commit_message>
<xml_diff>
--- a/spread.xlsx
+++ b/spread.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="227">
   <si>
     <t xml:space="preserve">xero</t>
   </si>
@@ -97,6 +97,9 @@
     <t xml:space="preserve">Marcin</t>
   </si>
   <si>
+    <t xml:space="preserve">Daga</t>
+  </si>
+  <si>
     <t xml:space="preserve">dupa</t>
   </si>
   <si>
@@ -403,250 +406,301 @@
     <t xml:space="preserve">Bridget Jones</t>
   </si>
   <si>
+    <t xml:space="preserve">barbie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">podwodne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tajni agenci</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zajebiste TEMPO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angry Birds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lesbijski Romans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wkurwiające Adiego</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niedźwiedzie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Johhnny Deepp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a czy wiedzieliście że?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">narkotyki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kot w butach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piekło Japończyków</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parkour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Musical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suda-core</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Europejski Tarantino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jaś fasola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zapomniane bajki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siostry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wkurwiona baba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japoński punk rock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mahlojki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">baba przebrana za chlopa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Western &lt; 3h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jetix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disney Channel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japonia w erze Muromachi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ktoś ucieka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dla koniar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mechy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nieśmiertelność</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anime reżyser live-action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O lataniu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mówiące zwierzątka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigma grindset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potwór Frankenstein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Współczesna japonia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koks dubbging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cringe disney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nie wierze że nie japoński</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faceci w Czerni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">powtórzenia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">podziemne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pamiętnik Księżniczki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Życiowe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gówniane anime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">piekło excela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gun Fu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">planszowkowe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kocham Amerykę!!!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taniec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supermoce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masochista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tańczące zwierzęta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">grzyby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gimby nie znajo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Narkotyki są złe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wielcy wynalazcy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Big pharma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Psychodeliczne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horrory2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horrory Nicholas Cage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dobry, słaby Adam Sandler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Współczesny Kopciuszek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ip man</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean girls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">djace do myslenia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imprezowe 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niezależne Anime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madagaskar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clanker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chuck Norris</t>
+  </si>
+  <si>
     <t xml:space="preserve">Moi mężowie</t>
   </si>
   <si>
-    <t xml:space="preserve">barbie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">podwodne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tajni agenci</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zajebiste TEMPO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Angry Birds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lesbijski Romans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wkurwiające Adiego</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niedźwiedzie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Johhnny Deepp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a czy wiedzieliście że?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">narkotyki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kot w butach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piekło Japończyków</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parkour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Musical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suda-core</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Europejski Tarantino</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jaś fasola</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zapomniane bajki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siostry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wkurwiona baba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Japoński punk rock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mahlojki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Simp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">baba przebrana za chlopa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Western &lt; 3h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jetix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disney Channel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Japonia w erze Muromachi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ktoś ucieka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dla koniar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mechy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nieśmiertelność</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anime reżyser live-action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O lataniu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mówiące zwierzątka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sigma grindset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Potwór Frankenstein</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Porno</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Współczesna japonia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Koks dubbging</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cringe disney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nie wierze że nie japoński</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faceci w Czerni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">powtórzenia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">podziemne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pamiętnik Księżniczki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Życiowe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gówniane anime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">piekło excela</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gun Fu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">planszowkowe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kocham Amerykę!!!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taniec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supermoce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masochista</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tańczące zwierzęta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grzyby</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gimby nie znajo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Narkotyki są złe</t>
+    <t xml:space="preserve">to jest na poidstawioe mangi:??+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kopcisz cd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rpg </t>
+  </si>
+  <si>
+    <t xml:space="preserve">hackowanie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moi mez 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bracia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wojenne </t>
+  </si>
+  <si>
+    <t xml:space="preserve">duuuuupa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jackie Chjanm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nicholas Cage 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">podróże w czasie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">polskie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">niewiadoma</t>
   </si>
   <si>
     <t xml:space="preserve">Surfowanie w animacji</t>
   </si>
   <si>
-    <t xml:space="preserve">Wielcy wynalazcy</t>
+    <t xml:space="preserve">Romans z babą robotem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simpy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asterix i Obelix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obcy są wśród nas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niszowe cartoon network</t>
   </si>
   <si>
     <t xml:space="preserve">kapitan bomba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Big pharma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Psychodeliczne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">horrory2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Horrory Nicholas Cage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dobry, słaby Adam Sandler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Współczesny Kopciuszek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ip man</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean girls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jackie Chan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">djace do myslenia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imprezowe 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niezależne Anime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Madagaskar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clanker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chuck Norris</t>
   </si>
 </sst>
 </file>
@@ -797,7 +851,7 @@
       <charset val="238"/>
     </font>
   </fonts>
-  <fills count="26">
+  <fills count="27">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -813,7 +867,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFD62E4E"/>
+        <bgColor rgb="FFBD0300"/>
       </patternFill>
     </fill>
     <fill>
@@ -948,6 +1002,12 @@
         <bgColor rgb="FF969696"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBD0300"/>
+        <bgColor rgb="FF800000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border diagonalUp="false" diagonalDown="false">
@@ -1121,6 +1181,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="26" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1174,10 +1238,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1200,7 +1260,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFCC00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FFBD0300"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFB09210"/>
@@ -1431,13 +1491,13 @@
     <tabColor rgb="FF00CC3E"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AB50"/>
+  <dimension ref="A1:AC53"/>
   <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="12.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="27.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.82"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="12.54"/>
@@ -1453,9 +1513,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="16.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="23.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="26.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="25" style="1" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="26.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="25.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="26.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="26.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="25.09"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1534,997 +1596,1031 @@
       <c r="Y1" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="29" t="s">
+      <c r="AA1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="30"/>
+      <c r="AB1" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="31"/>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="30"/>
-      <c r="B2" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="30" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="32" t="s">
+      <c r="C2" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="H2" s="32"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="29"/>
-      <c r="Q2" s="29"/>
-      <c r="R2" s="29"/>
-      <c r="Z2" s="34" t="s">
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="AA2" s="29" t="s">
+      <c r="H2" s="33"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="34"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="30"/>
+      <c r="Q2" s="30"/>
+      <c r="R2" s="30"/>
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB2" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="AB2" s="30" t="s">
-        <v>31</v>
+      <c r="AC2" s="31" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="32"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="32"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="32"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="29"/>
-      <c r="R3" s="29"/>
-      <c r="Z3" s="34"/>
-      <c r="AA3" s="29" t="s">
+      <c r="B3" s="33"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="33"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="33"/>
+      <c r="P3" s="30"/>
+      <c r="Q3" s="30"/>
+      <c r="R3" s="30"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="AB3" s="30" t="s">
-        <v>33</v>
+      <c r="AC3" s="31" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="32"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="29"/>
-      <c r="R4" s="29"/>
-      <c r="Z4" s="34"/>
-      <c r="AA4" s="29" t="s">
+      <c r="B4" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="33"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="34"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="30"/>
+      <c r="R4" s="30"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="AB4" s="30" t="s">
-        <v>35</v>
+      <c r="AC4" s="31" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="32"/>
-      <c r="L5" s="32"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="32"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="29"/>
-      <c r="R5" s="29"/>
-      <c r="Z5" s="34"/>
-      <c r="AA5" s="29" t="s">
+      <c r="B5" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="33"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="30"/>
+      <c r="R5" s="30"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3"/>
+      <c r="AB5" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="AB5" s="30" t="s">
-        <v>37</v>
+      <c r="AC5" s="31" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="32"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="M6" s="30"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="32" t="s">
+      <c r="B6" s="33"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="33"/>
+      <c r="L6" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="P6" s="29"/>
-      <c r="Q6" s="29"/>
-      <c r="R6" s="29"/>
-      <c r="Z6" s="34"/>
-      <c r="AA6" s="29" t="s">
+      <c r="M6" s="31"/>
+      <c r="N6" s="34"/>
+      <c r="O6" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="P6" s="30"/>
+      <c r="Q6" s="30"/>
+      <c r="R6" s="30"/>
+      <c r="Z6" s="3"/>
+      <c r="AA6" s="3"/>
+      <c r="AB6" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="AB6" s="30" t="s">
-        <v>40</v>
+      <c r="AC6" s="31" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="32"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="J7" s="30"/>
-      <c r="K7" s="32"/>
-      <c r="L7" s="32"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="33"/>
-      <c r="O7" s="32"/>
-      <c r="P7" s="29"/>
-      <c r="Q7" s="29"/>
-      <c r="R7" s="29"/>
-      <c r="Z7" s="34"/>
-      <c r="AA7" s="29" t="s">
+      <c r="B7" s="33"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" s="31"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="33"/>
+      <c r="P7" s="30"/>
+      <c r="Q7" s="30"/>
+      <c r="R7" s="30"/>
+      <c r="Z7" s="3"/>
+      <c r="AA7" s="3"/>
+      <c r="AB7" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="AB7" s="30" t="s">
+      <c r="AC7" s="31" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="33"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="31" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="32"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="30"/>
-      <c r="N8" s="33"/>
-      <c r="O8" s="32"/>
-      <c r="P8" s="29"/>
-      <c r="Q8" s="29"/>
-      <c r="R8" s="29"/>
-      <c r="Z8" s="34"/>
-      <c r="AA8" s="29" t="s">
+      <c r="K8" s="33"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="34"/>
+      <c r="O8" s="33"/>
+      <c r="P8" s="30"/>
+      <c r="Q8" s="30"/>
+      <c r="R8" s="30"/>
+      <c r="Z8" s="3"/>
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="AB8" s="30" t="s">
-        <v>43</v>
+      <c r="AC8" s="31" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="32"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="F9" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="J9" s="30"/>
-      <c r="K9" s="32"/>
-      <c r="L9" s="32"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="33"/>
-      <c r="O9" s="32"/>
-      <c r="P9" s="29"/>
-      <c r="Q9" s="29"/>
-      <c r="R9" s="29"/>
-      <c r="Z9" s="34"/>
-      <c r="AA9" s="29" t="s">
+      <c r="B9" s="33"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="F9" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="31"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="33"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="33"/>
+      <c r="P9" s="30"/>
+      <c r="Q9" s="30"/>
+      <c r="R9" s="30"/>
+      <c r="Z9" s="3"/>
+      <c r="AA9" s="3"/>
+      <c r="AB9" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="AB9" s="30" t="s">
+      <c r="AC9" s="31" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="33"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="32"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="32"/>
-      <c r="L10" s="32"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="33"/>
-      <c r="O10" s="32"/>
-      <c r="P10" s="29"/>
-      <c r="Q10" s="29"/>
-      <c r="R10" s="29"/>
-      <c r="Z10" s="34"/>
-      <c r="AA10" s="29" t="s">
+      <c r="G10" s="33"/>
+      <c r="H10" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="33"/>
+      <c r="P10" s="30"/>
+      <c r="Q10" s="30"/>
+      <c r="R10" s="30"/>
+      <c r="Z10" s="3"/>
+      <c r="AA10" s="3"/>
+      <c r="AB10" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="AB10" s="30" t="s">
+      <c r="AC10" s="31" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="33"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="31"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="32"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="F11" s="30"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="I11" s="30"/>
-      <c r="J11" s="30"/>
-      <c r="K11" s="32"/>
-      <c r="L11" s="32"/>
-      <c r="M11" s="30"/>
-      <c r="N11" s="33"/>
-      <c r="O11" s="32"/>
-      <c r="P11" s="29"/>
-      <c r="Q11" s="29"/>
-      <c r="R11" s="29"/>
-      <c r="Z11" s="34"/>
-      <c r="AA11" s="35" t="s">
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="33"/>
+      <c r="L11" s="33"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="34"/>
+      <c r="O11" s="33"/>
+      <c r="P11" s="30"/>
+      <c r="Q11" s="30"/>
+      <c r="R11" s="30"/>
+      <c r="Z11" s="3"/>
+      <c r="AA11" s="3"/>
+      <c r="AB11" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="AB11" s="30" t="s">
-        <v>49</v>
+      <c r="AC11" s="31" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="32"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" s="30"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="32"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="33"/>
-      <c r="O12" s="32"/>
-      <c r="P12" s="29"/>
-      <c r="Q12" s="29"/>
-      <c r="R12" s="29"/>
-      <c r="Z12" s="34"/>
-      <c r="AA12" s="37" t="s">
+      <c r="B12" s="33"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="31"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="34"/>
+      <c r="O12" s="33"/>
+      <c r="P12" s="30"/>
+      <c r="Q12" s="30"/>
+      <c r="R12" s="30"/>
+      <c r="Z12" s="3"/>
+      <c r="AA12" s="3"/>
+      <c r="AB12" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="AB12" s="30" t="s">
-        <v>51</v>
+      <c r="AC12" s="31" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="32"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="I13" s="30" t="s">
+      <c r="B13" s="33"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="J13" s="30"/>
-      <c r="K13" s="32" t="s">
+      <c r="I13" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="L13" s="32"/>
-      <c r="M13" s="30"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="32"/>
-      <c r="P13" s="29"/>
-      <c r="Q13" s="29"/>
-      <c r="R13" s="29"/>
-      <c r="Z13" s="34"/>
-      <c r="AA13" s="37" t="s">
+      <c r="J13" s="31"/>
+      <c r="K13" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="L13" s="33"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="34"/>
+      <c r="O13" s="33"/>
+      <c r="P13" s="30"/>
+      <c r="Q13" s="30"/>
+      <c r="R13" s="30"/>
+      <c r="Z13" s="3"/>
+      <c r="AA13" s="3"/>
+      <c r="AB13" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="AB13" s="30" t="s">
-        <v>55</v>
+      <c r="AC13" s="31" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="F14" s="30"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="I14" s="30"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="32"/>
-      <c r="L14" s="32" t="s">
+      <c r="A14" s="31"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="M14" s="30"/>
-      <c r="N14" s="33"/>
-      <c r="O14" s="32"/>
-      <c r="P14" s="29"/>
-      <c r="Q14" s="29"/>
-      <c r="R14" s="29"/>
-      <c r="Z14" s="34"/>
-      <c r="AA14" s="35" t="s">
+      <c r="F14" s="31"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="33"/>
+      <c r="L14" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="M14" s="31"/>
+      <c r="N14" s="34"/>
+      <c r="O14" s="33"/>
+      <c r="P14" s="30"/>
+      <c r="Q14" s="30"/>
+      <c r="R14" s="30"/>
+      <c r="Z14" s="3"/>
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="AB14" s="30" t="s">
-        <v>58</v>
+      <c r="AC14" s="31" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="30"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="I15" s="30" t="s">
+      <c r="A15" s="31"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="J15" s="30"/>
-      <c r="K15" s="32"/>
-      <c r="L15" s="32"/>
-      <c r="M15" s="30"/>
-      <c r="N15" s="33" t="s">
+      <c r="I15" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="O15" s="32"/>
-      <c r="P15" s="35"/>
-      <c r="Q15" s="35"/>
-      <c r="R15" s="35"/>
-      <c r="Z15" s="34"/>
-      <c r="AA15" s="38" t="s">
+      <c r="J15" s="31"/>
+      <c r="K15" s="33"/>
+      <c r="L15" s="33"/>
+      <c r="M15" s="31"/>
+      <c r="N15" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="O15" s="33"/>
+      <c r="P15" s="36"/>
+      <c r="Q15" s="36"/>
+      <c r="R15" s="36"/>
+      <c r="Z15" s="3"/>
+      <c r="AA15" s="3"/>
+      <c r="AB15" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="AB15" s="30" t="s">
+      <c r="AC15" s="31" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="31"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="34"/>
+      <c r="O16" s="33"/>
+      <c r="Q16" s="36"/>
+      <c r="R16" s="36"/>
+      <c r="Z16" s="3"/>
+      <c r="AA16" s="3"/>
+      <c r="AB16" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC16" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="33"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="I17" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="J17" s="31"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="33"/>
+      <c r="M17" s="31"/>
+      <c r="N17" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="O17" s="33"/>
+      <c r="Q17" s="36"/>
+      <c r="R17" s="36"/>
+      <c r="Z17" s="3"/>
+      <c r="AA17" s="3"/>
+      <c r="AB17" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC17" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="33"/>
+      <c r="C18" s="31"/>
+      <c r="F18" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="33"/>
+      <c r="L18" s="33"/>
+      <c r="M18" s="31"/>
+      <c r="N18" s="34"/>
+      <c r="O18" s="33"/>
+      <c r="Q18" s="36"/>
+      <c r="R18" s="36"/>
+      <c r="Z18" s="3"/>
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC18" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="31"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="F19" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="I19" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="J19" s="31"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="34"/>
+      <c r="O19" s="33"/>
+      <c r="P19" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q19" s="36"/>
+      <c r="R19" s="36"/>
+      <c r="Z19" s="3"/>
+      <c r="AA19" s="3"/>
+      <c r="AB19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC19" s="31" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="33"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="31"/>
+      <c r="N20" s="34"/>
+      <c r="O20" s="33"/>
+      <c r="Q20" s="36"/>
+      <c r="R20" s="36"/>
+      <c r="Z20" s="3"/>
+      <c r="AA20" s="3"/>
+      <c r="AB20" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="31" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="33"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="31"/>
+      <c r="N21" s="34" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="30"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="33"/>
-      <c r="O16" s="32"/>
-      <c r="Q16" s="35"/>
-      <c r="R16" s="35"/>
-      <c r="Z16" s="34"/>
-      <c r="AA16" s="38" t="s">
-        <v>5</v>
-      </c>
-      <c r="AB16" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="32"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="G17" s="32"/>
-      <c r="H17" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="I17" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="J17" s="30"/>
-      <c r="K17" s="32"/>
-      <c r="L17" s="32"/>
-      <c r="M17" s="30"/>
-      <c r="N17" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="O17" s="32"/>
-      <c r="Q17" s="35"/>
-      <c r="R17" s="35"/>
-      <c r="Z17" s="34"/>
-      <c r="AA17" s="35" t="s">
-        <v>3</v>
-      </c>
-      <c r="AB17" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="32"/>
-      <c r="C18" s="30"/>
-      <c r="F18" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="30"/>
-      <c r="N18" s="33"/>
-      <c r="O18" s="32"/>
-      <c r="Q18" s="35"/>
-      <c r="R18" s="35"/>
-      <c r="Z18" s="34"/>
-      <c r="AA18" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="AB18" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="F19" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="I19" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="J19" s="30"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="30"/>
-      <c r="N19" s="33"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q19" s="35"/>
-      <c r="R19" s="35"/>
-      <c r="Z19" s="34"/>
-      <c r="AA19" s="3" t="s">
+      <c r="O21" s="33"/>
+      <c r="Q21" s="36"/>
+      <c r="R21" s="36"/>
+      <c r="Z21" s="3"/>
+      <c r="AA21" s="3"/>
+      <c r="AB21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC21" s="31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="31"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="31"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="31"/>
+      <c r="N22" s="34"/>
+      <c r="O22" s="33"/>
+      <c r="Q22" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="R22" s="36"/>
+      <c r="Z22" s="3"/>
+      <c r="AA22" s="3"/>
+      <c r="AB22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC22" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="31"/>
+      <c r="B23" s="33"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="J23" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="31"/>
+      <c r="N23" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="O23" s="33"/>
+      <c r="Q23" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="R23" s="36"/>
+      <c r="Z23" s="3"/>
+      <c r="AA23" s="3"/>
+      <c r="AB23" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D24" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="N24" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="P24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q24" s="36"/>
+      <c r="R24" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="S24" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z24" s="3"/>
+      <c r="AA24" s="3"/>
+      <c r="AB24" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="AB19" s="30" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="32"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="32"/>
-      <c r="L20" s="32"/>
-      <c r="M20" s="30"/>
-      <c r="N20" s="33"/>
-      <c r="O20" s="32"/>
-      <c r="Q20" s="35"/>
-      <c r="R20" s="35"/>
-      <c r="Z20" s="34"/>
-      <c r="AA20" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="30" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="32"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="30"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="30"/>
-      <c r="N21" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="O21" s="32"/>
-      <c r="Q21" s="35"/>
-      <c r="R21" s="35"/>
-      <c r="Z21" s="34"/>
-      <c r="AA21" s="3" t="s">
+      <c r="AC24" s="31" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="34"/>
+      <c r="D25" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="N25" s="34"/>
+      <c r="Q25" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="R25" s="36"/>
+      <c r="Z25" s="3"/>
+      <c r="AA25" s="3"/>
+      <c r="AB25" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="AB21" s="30" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="F22" s="30"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="32"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="K22" s="32"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="30"/>
-      <c r="N22" s="33"/>
-      <c r="O22" s="32"/>
-      <c r="Q22" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="R22" s="35"/>
-      <c r="Z22" s="34"/>
-      <c r="AA22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AB22" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="30"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="32"/>
-      <c r="I23" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="J23" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="K23" s="32"/>
-      <c r="L23" s="32"/>
-      <c r="M23" s="30"/>
-      <c r="N23" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="O23" s="32"/>
-      <c r="Q23" s="35" t="s">
-        <v>79</v>
-      </c>
-      <c r="R23" s="35"/>
-      <c r="Z23" s="34"/>
-      <c r="AA23" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D24" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="N24" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="P24" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q24" s="35"/>
-      <c r="R24" s="35" t="s">
-        <v>81</v>
-      </c>
-      <c r="S24" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="Z24" s="34"/>
-      <c r="AA24" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="AB24" s="30" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="33"/>
-      <c r="D25" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="M25" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="N25" s="33"/>
-      <c r="Q25" s="35" t="s">
-        <v>88</v>
-      </c>
-      <c r="R25" s="35"/>
-      <c r="Z25" s="34"/>
-      <c r="AA25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AB25" s="3" t="s">
-        <v>89</v>
+      <c r="AC25" s="3" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="33"/>
+      <c r="A26" s="34"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q26" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="R26" s="35"/>
-      <c r="Z26" s="34"/>
-      <c r="AA26" s="3" t="s">
+      <c r="Q26" s="36" t="s">
+        <v>94</v>
+      </c>
+      <c r="R26" s="36"/>
+      <c r="Z26" s="3"/>
+      <c r="AA26" s="3"/>
+      <c r="AB26" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="AB26" s="30" t="s">
-        <v>94</v>
+      <c r="AC26" s="31" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="33"/>
+      <c r="A27" s="34"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="I27" s="30" t="s">
-        <v>60</v>
+        <v>96</v>
+      </c>
+      <c r="I27" s="31" t="s">
+        <v>61</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q27" s="35" t="s">
-        <v>96</v>
-      </c>
-      <c r="R27" s="35"/>
+        <v>93</v>
+      </c>
+      <c r="Q27" s="36" t="s">
+        <v>97</v>
+      </c>
+      <c r="R27" s="36"/>
       <c r="T27" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="Z27" s="34"/>
-      <c r="AA27" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z27" s="3"/>
+      <c r="AA27" s="3"/>
+      <c r="AB27" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="AB27" s="3" t="s">
-        <v>98</v>
+      <c r="AC27" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q28" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="R28" s="35"/>
+      <c r="Q28" s="36" t="s">
+        <v>100</v>
+      </c>
+      <c r="R28" s="36"/>
       <c r="T28" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="U28" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="Z28" s="34"/>
-      <c r="AA28" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="Z28" s="3"/>
+      <c r="AA28" s="3"/>
+      <c r="AB28" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="AB28" s="3" t="s">
-        <v>102</v>
+      <c r="AC28" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J29" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="Q29" s="35" t="s">
         <v>104</v>
       </c>
-      <c r="R29" s="35"/>
-      <c r="Z29" s="34"/>
-      <c r="AA29" s="3" t="s">
+      <c r="Q29" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="R29" s="36"/>
+      <c r="Z29" s="3"/>
+      <c r="AA29" s="3"/>
+      <c r="AB29" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="AB29" s="30" t="s">
-        <v>105</v>
+      <c r="AC29" s="31" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D30" s="3"/>
       <c r="E30" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q30" s="35" t="s">
-        <v>107</v>
-      </c>
-      <c r="R30" s="35"/>
+        <v>66</v>
+      </c>
+      <c r="Q30" s="36" t="s">
+        <v>108</v>
+      </c>
+      <c r="R30" s="36"/>
       <c r="U30" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z30" s="34"/>
-      <c r="AA30" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="Z30" s="3"/>
+      <c r="AA30" s="3"/>
+      <c r="AB30" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="AB30" s="40" t="s">
-        <v>109</v>
+      <c r="AC30" s="41" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="Q31" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="R31" s="35"/>
+      <c r="Q31" s="36" t="s">
+        <v>113</v>
+      </c>
+      <c r="R31" s="36"/>
       <c r="V31" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="Z31" s="34"/>
-      <c r="AA31" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="Z31" s="3"/>
+      <c r="AA31" s="3"/>
+      <c r="AB31" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="AB31" s="3" t="s">
-        <v>114</v>
+      <c r="AC31" s="3" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C32" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="I32" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q32" s="35" t="s">
-        <v>93</v>
+        <v>117</v>
+      </c>
+      <c r="I32" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q32" s="36" t="s">
+        <v>94</v>
       </c>
       <c r="T32" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="Z32" s="34"/>
-      <c r="AA32" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z32" s="3"/>
+      <c r="AA32" s="3"/>
+      <c r="AB32" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="AB32" s="3" t="s">
-        <v>118</v>
+      <c r="AC32" s="3" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D33" s="3"/>
       <c r="I33" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="N33" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="P33" s="35"/>
-      <c r="Q33" s="35" t="s">
-        <v>93</v>
+        <v>87</v>
+      </c>
+      <c r="N33" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="P33" s="36"/>
+      <c r="Q33" s="36" t="s">
+        <v>94</v>
       </c>
       <c r="T33" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="Z33" s="34"/>
-      <c r="AA33" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z33" s="3"/>
+      <c r="AA33" s="3"/>
+      <c r="AB33" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="AB33" s="3" t="s">
-        <v>120</v>
+      <c r="AC33" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="N34" s="33"/>
-      <c r="P34" s="35"/>
+        <v>104</v>
+      </c>
+      <c r="N34" s="34"/>
+      <c r="P34" s="36"/>
       <c r="T34" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z34" s="34"/>
-      <c r="AA34" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z34" s="3"/>
+      <c r="AA34" s="3"/>
+      <c r="AB34" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="AB34" s="3" t="s">
-        <v>124</v>
+      <c r="AC34" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D35" s="30"/>
+        <v>126</v>
+      </c>
+      <c r="D35" s="31"/>
       <c r="E35" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="P35" s="35"/>
+        <v>66</v>
+      </c>
+      <c r="P35" s="36"/>
       <c r="Q35" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="U35" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="Z35" s="34"/>
-      <c r="AA35" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="Z35" s="3"/>
+      <c r="AA35" s="3"/>
+      <c r="AB35" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB35" s="3" t="s">
+      <c r="AC35" s="3" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B36" s="41"/>
-      <c r="F36" s="0"/>
-      <c r="G36" s="41"/>
-      <c r="H36" s="41"/>
+        <v>126</v>
+      </c>
+      <c r="B36" s="42"/>
+      <c r="G36" s="42"/>
+      <c r="H36" s="42"/>
       <c r="I36" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K36" s="41"/>
-      <c r="L36" s="41"/>
-      <c r="N36" s="40"/>
-      <c r="O36" s="41"/>
+      <c r="K36" s="42"/>
+      <c r="L36" s="42"/>
+      <c r="N36" s="41"/>
+      <c r="O36" s="42"/>
       <c r="Q36" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="T36" s="40" t="s">
-        <v>100</v>
-      </c>
-      <c r="Z36" s="34"/>
-      <c r="AA36" s="39" t="s">
+        <v>108</v>
+      </c>
+      <c r="T36" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z36" s="3"/>
+      <c r="AA36" s="3"/>
+      <c r="AB36" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="AB36" s="3" t="s">
+      <c r="AC36" s="3" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>131</v>
@@ -2532,9 +2628,9 @@
       <c r="E37" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="F37" s="42"/>
-      <c r="I37" s="30" t="s">
-        <v>41</v>
+      <c r="F37" s="43"/>
+      <c r="I37" s="31" t="s">
+        <v>42</v>
       </c>
       <c r="N37" s="3" t="s">
         <v>133</v>
@@ -2548,17 +2644,18 @@
       <c r="U37" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="Z37" s="34"/>
-      <c r="AA37" s="39" t="s">
+      <c r="Z37" s="3"/>
+      <c r="AA37" s="3"/>
+      <c r="AB37" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="AB37" s="3" t="s">
+      <c r="AC37" s="3" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>138</v>
@@ -2567,25 +2664,23 @@
         <v>131</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="T38" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="U38" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="Z38" s="34"/>
-      <c r="AA38" s="3" t="s">
+      <c r="Z38" s="3"/>
+      <c r="AA38" s="3"/>
+      <c r="AB38" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="AB38" s="30" t="s">
+      <c r="AC38" s="31" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>138</v>
@@ -2593,27 +2688,25 @@
       <c r="D39" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="F39" s="42"/>
+      <c r="F39" s="43"/>
       <c r="Q39" s="3" t="s">
         <v>142</v>
       </c>
       <c r="T39" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="U39" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="Z39" s="34"/>
-      <c r="AA39" s="3" t="s">
+      <c r="Z39" s="3"/>
+      <c r="AA39" s="3"/>
+      <c r="AB39" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="AB39" s="30" t="s">
+      <c r="AC39" s="31" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>138</v>
@@ -2634,22 +2727,23 @@
         <v>142</v>
       </c>
       <c r="T40" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="W40" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="Z40" s="34"/>
-      <c r="AA40" s="3" t="s">
+      <c r="Z40" s="3"/>
+      <c r="AA40" s="3"/>
+      <c r="AB40" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="AB40" s="3" t="s">
+      <c r="AC40" s="3" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>138</v>
@@ -2658,7 +2752,7 @@
         <v>150</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>147</v>
@@ -2667,22 +2761,20 @@
         <v>151</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q41" s="3" t="s">
         <v>152</v>
       </c>
       <c r="T41" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="U41" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="Z41" s="34"/>
-      <c r="AA41" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z41" s="3"/>
+      <c r="AA41" s="3"/>
+      <c r="AB41" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="AB41" s="30" t="s">
+      <c r="AC41" s="31" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2696,9 +2788,9 @@
       <c r="E42" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F42" s="42"/>
-      <c r="Q42" s="35" t="s">
-        <v>104</v>
+      <c r="F42" s="43"/>
+      <c r="Q42" s="36" t="s">
+        <v>105</v>
       </c>
       <c r="T42" s="3" t="s">
         <v>143</v>
@@ -2710,11 +2802,12 @@
         <v>158</v>
       </c>
       <c r="Y42" s="3"/>
-      <c r="Z42" s="34"/>
-      <c r="AA42" s="3" t="s">
+      <c r="Z42" s="3"/>
+      <c r="AA42" s="3"/>
+      <c r="AB42" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="AB42" s="3" t="s">
+      <c r="AC42" s="3" t="s">
         <v>159</v>
       </c>
     </row>
@@ -2738,7 +2831,7 @@
         <v>164</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="T43" s="3" t="s">
         <v>165</v>
@@ -2746,11 +2839,12 @@
       <c r="W43" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="Z43" s="34"/>
-      <c r="AA43" s="1" t="s">
+      <c r="Z43" s="3"/>
+      <c r="AA43" s="3"/>
+      <c r="AB43" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AB43" s="3" t="s">
+      <c r="AC43" s="3" t="s">
         <v>166</v>
       </c>
     </row>
@@ -2768,10 +2862,10 @@
         <v>147</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="Q44" s="35" t="s">
         <v>104</v>
+      </c>
+      <c r="Q44" s="36" t="s">
+        <v>105</v>
       </c>
       <c r="T44" s="3"/>
       <c r="W44" s="1" t="s">
@@ -2780,11 +2874,12 @@
       <c r="X44" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="Z44" s="34"/>
-      <c r="AA44" s="1" t="s">
+      <c r="Z44" s="3"/>
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="AB44" s="1" t="s">
+      <c r="AC44" s="1" t="s">
         <v>171</v>
       </c>
     </row>
@@ -2792,7 +2887,7 @@
       <c r="A45" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C45" s="40" t="s">
+      <c r="C45" s="41" t="s">
         <v>161</v>
       </c>
       <c r="D45" s="1" t="s">
@@ -2807,23 +2902,24 @@
       <c r="I45" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="J45" s="40" t="s">
-        <v>103</v>
+      <c r="J45" s="41" t="s">
+        <v>104</v>
       </c>
       <c r="M45" s="1" t="s">
         <v>176</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="W45" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="Z45" s="34"/>
-      <c r="AA45" s="1" t="s">
+      <c r="Z45" s="3"/>
+      <c r="AA45" s="3"/>
+      <c r="AB45" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AB45" s="3" t="s">
+      <c r="AC45" s="3" t="s">
         <v>178</v>
       </c>
     </row>
@@ -2831,7 +2927,7 @@
       <c r="A46" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="C46" s="40" t="s">
+      <c r="C46" s="41" t="s">
         <v>161</v>
       </c>
       <c r="D46" s="3" t="s">
@@ -2840,10 +2936,10 @@
       <c r="W46" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="AA46" s="3" t="s">
+      <c r="AB46" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="AB46" s="3" t="s">
+      <c r="AC46" s="3" t="s">
         <v>181</v>
       </c>
     </row>
@@ -2864,15 +2960,15 @@
         <v>184</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q47" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="AA47" s="1" t="s">
+      <c r="AB47" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AB47" s="1" t="s">
+      <c r="AC47" s="1" t="s">
         <v>186</v>
       </c>
     </row>
@@ -2886,43 +2982,38 @@
       <c r="D48" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>190</v>
-      </c>
       <c r="F48" s="3" t="s">
         <v>147</v>
       </c>
       <c r="I48" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q48" s="0"/>
+      <c r="T48" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="Q48" s="1" t="s">
+      <c r="X48" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="T48" s="3" t="s">
+      <c r="AB48" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AC48" s="37" t="s">
         <v>193</v>
-      </c>
-      <c r="X48" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="AA48" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB48" s="36" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>161</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="I49" s="3" t="s">
         <v>129</v>
@@ -2931,22 +3022,19 @@
         <v>133</v>
       </c>
       <c r="Q49" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="V49" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="X49" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="Y49" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AA49" s="1" t="s">
+      <c r="AB49" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AB49" s="42" t="s">
-        <v>202</v>
+      <c r="AC49" s="43" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2954,31 +3042,124 @@
         <v>179</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="I50" s="43" t="s">
+      <c r="I50" s="3" t="s">
         <v>151</v>
       </c>
       <c r="Q50" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="T50" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="Y50" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="AB50" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC50" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="T50" s="43" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="U50" s="43" t="s">
-        <v>127</v>
-      </c>
-      <c r="Y50" s="1" t="s">
+      <c r="E51" s="1" t="s">
         <v>208</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q51" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="T51" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="U51" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="W51" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="Y51" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="AA51" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="AB51" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC51" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q52" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y52" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="AB52" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC52" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="Z53" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB53" s="40" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC53" s="1" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>